<commit_message>
docs(ai-media-education-dx): apply Padiem provider identity
Apply final provider identity 파디엠 (PADIEM) to the Business 35 customer package.

- Proposal: cover shows '제공: 파디엠'; all footers '파디엠 · DRAFT'; last page adds '제공 및 계약 주체: 파디엠' + pricing/legal-review closing
- One-page: '제공: 파디엠' in header, footer '파디엠 · DRAFT'
- Questionnaire: repeating page header '파디엠 · AI 업무전환 진단 질문지' + [N/3]
- Quote workbook: supplier/contracting/issuer = 파디엠; business details marked '발송 전 공식 사업자 정보 입력 필요' (no invented numbers)
- Meeting script / emails: Padiem self-intro, sender '파디엠 · AI 업무전환 프로그램'
- Internal docs (README/CHECKLIST/SOURCE_MAPPING/VISUAL_QA/REFERENCE_COMPARISON): FINAL_IDENTITY_DECIDED · PROVIDER 파디엠 · CONTRACTING_ENTITY 파디엠 · BUSINESS_DETAILS_VERIFICATION_PENDING
- Pricing/product scope unchanged (A/B1/B2/C)
- AI Revenue Lab not shown as contracting entity

Validation: ALL CHECKS PASSED; git diff --check clean; PDF 10/1/3; renders 14; XLSX 9 sheets.

Refs #359.
</commit_message>
<xml_diff>
--- a/docs/commercial/business-35-ai-media-education-dx/customer-package/Business35_Pilot_Quote_Template.xlsx
+++ b/docs/commercial/business-35-ai-media-education-dx/customer-package/Business35_Pilot_Quote_Template.xlsx
@@ -100,7 +100,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -122,24 +122,58 @@
         <color rgb="00B0B7C0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B7C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B7C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B7C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B7C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B7C0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B7C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -518,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -536,7 +570,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>CUSTOMER-FACING MASTER · FINAL IDENTITY REQUIRED · LEGAL REVIEW REQUIRED · NOT YET SENT</t>
+          <t>공급자: 파디엠</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
@@ -544,98 +578,118 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>제안 제공자 정보는 발송 전 최종 확정</t>
+          <t>제공 및 계약 주체: 파디엠</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>견적 발행 주체: 파디엠</t>
+        </is>
+      </c>
       <c r="B4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>사용 방법</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>각 Offer sheet에 금액(원, VAT 별도)과 인원·기간을 입력합니다.</t>
-        </is>
-      </c>
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>계산</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>공급가액 / VAT(10%) / 합계가 자동 계산됩니다. 지급 단계(착수금 50%·잔금 50%)를 확인합니다.</t>
+          <t>사용 방법</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>각 Offer sheet에 금액(원, VAT 별도)과 인원·기간을 입력합니다.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>경고</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>표준 가격 범위를 벗어나는 금액을 입력하면 해당 셀에 경고가 표시됩니다.</t>
+          <t>계산</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>공급가액 / VAT(10%) / 합계가 자동 계산됩니다. 지급 단계(착수금 50%·잔금 50%)를 확인합니다.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>표준 가격</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>A 진단 워크숍 초기형 300만–500만원 · A 확장형 500만–800만원 · B1 디자인 파트너 1,000만–1,500만원 · B2 표준 1,500만–2,500만원 · C 운영 자문 월 300만–600만원</t>
+          <t>경고</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>표준 가격 범위를 벗어나는 금액을 입력하면 해당 셀에 경고가 표시됩니다.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>상태</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>견적 검토 템플릿 — 계약 확정 문서가 아닙니다.</t>
+          <t>표준 가격</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>A 진단 워크숍 초기형 300만–500만원 · A 확장형 500만–800만원 · B1 디자인 파트너 1,000만–1,500만원 · B2 표준 1,500만–2,500만원 · C 운영 자문 월 300만–600만원</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>상태</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>견적 검토 템플릿 — 계약 확정 문서가 아닙니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>가격 정책</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>시장 검증 전 자사 가격 가설 · 범위와 인원·기간에 따라 최종 견적 · VAT 조건은 최종 견적서에서 확정</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="6" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>주의</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>발송 전 공식 사업자 정보 입력 필요 (사업자등록번호·대표자·주소·연락처·계좌).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>주의</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>본 템플릿은 고객에게 발송 전 최종 승인과 전문 법률·계약 검토가 필요합니다.</t>
         </is>
@@ -1576,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1593,76 +1647,147 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>견적 준비자</t>
+          <t>제공 및 계약 주체</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>[이름/직책]</t>
+          <t>파디엠</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>견적 승인자 (제공자)</t>
+          <t>공급자</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>[이름/직책]</t>
+          <t>파디엠</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>고객 승인자</t>
+          <t>사업자등록번호</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>[직책]</t>
+          <t>발송 전 공식 사업자 정보 입력 필요</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>승인일</t>
+          <t>대표자·주소·연락처</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>[YYYY-MM-DD]</t>
+          <t>발송 전 공식 사업자 정보 입력 필요</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>상태</t>
+          <t>입금 계좌 (은행명·예금주)</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>견적 검토 중 (계약 확정 아님)</t>
+          <t>발송 전 공식 사업자 정보 입력 필요</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
+          <t>견적 준비자</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>[이름/직책]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>견적 승인자 (제공자)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>[이름/직책]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>고객 승인자</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>[직책]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>승인일</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>[YYYY-MM-DD]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>상태</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>견적 검토 중 (계약 확정 아님)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
           <t>법률·계약 검토</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>REQUIRED — DRAFT · PROFESSIONAL LEGAL REVIEW REQUIRED</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>안내: 사업자등록번호·대표자·주소·연락처·계좌 정보는 발송 전 공식 확인 후 입력합니다.</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A15:B15"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>